<commit_message>
data: clear Config.xlsx data rows, keep headers only
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/Data/Config.xlsx
+++ b/project/Data/Config.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Settings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Constants" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Assets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constants" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -445,112 +445,18 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>FeatureName</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>TypesDemo</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MaxItems</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>42</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Threshold</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3.14</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>double</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>IsEnabled</t>
-        </is>
-      </c>
-      <c r="B5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CutoffDate</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>46022</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DateOnly — date only, time is 00:00:00</t>
-        </is>
-      </c>
+      <c r="B6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>ScheduledAt</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>45823.39583333334</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DateTime — has time component</t>
-        </is>
-      </c>
+      <c r="B7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>DailyRunTime</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TimeOnly — time only, no date</t>
-        </is>
-      </c>
+      <c r="B8" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -583,110 +489,20 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Pi</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3.14159</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>double — mathematical constant</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MaxRetryNumber</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>StrictMode</t>
-        </is>
-      </c>
-      <c r="B4" t="b">
-        <v>0</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-    </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ExpiresOn</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>46023</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>DateOnly</t>
-        </is>
-      </c>
+      <c r="B5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CreatedAt</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>45352.5</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
+      <c r="B6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>WindowOpen</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>TimeOnly</t>
-        </is>
-      </c>
+      <c r="B7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>WindowClose</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>0.7291666666666666</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>TimeOnly</t>
-        </is>
-      </c>
+      <c r="B8" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>